<commit_message>
csv css en index updates
csv css en index updates
</commit_message>
<xml_diff>
--- a/CSV/Ancient City.xlsx
+++ b/CSV/Ancient City.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/willem/Documents/GitHub/friend-zone/CSV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3A09DA-E683-004D-A0DE-6729AF00C9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A63BAA-E533-284E-9C53-A6C87E1FDC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9620" windowWidth="11480" windowHeight="9980" xr2:uid="{EF5563DD-86E3-44AF-B99F-9E11ACF57133}"/>
   </bookViews>
@@ -426,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2061EA4-28D3-4349-9580-4EA67BE3ACE4}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -548,10 +548,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>2824</v>
+        <v>-744</v>
       </c>
       <c r="C11">
-        <v>-3320</v>
+        <v>-184</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -559,10 +559,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>2856</v>
+        <v>2824</v>
       </c>
       <c r="C12">
-        <v>-3704</v>
+        <v>-3320</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -570,10 +570,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>3592</v>
+        <v>2856</v>
       </c>
       <c r="C13">
-        <v>-1800</v>
+        <v>-3704</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -581,10 +581,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>3928</v>
+        <v>3592</v>
       </c>
       <c r="C14">
-        <v>-2216</v>
+        <v>-1800</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -592,10 +592,10 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>3960</v>
+        <v>3928</v>
       </c>
       <c r="C15">
-        <v>-3000</v>
+        <v>-2216</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -603,9 +603,20 @@
         <v>15</v>
       </c>
       <c r="B16">
+        <v>3960</v>
+      </c>
+      <c r="C16">
+        <v>-3000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
         <v>5128</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>2920</v>
       </c>
     </row>

</xml_diff>